<commit_message>
update Cancelar task and add Extraer imagenes
</commit_message>
<xml_diff>
--- a/Automatismo/Automatizaciones/Cancelar task/cancel.xlsx
+++ b/Automatismo/Automatizaciones/Cancelar task/cancel.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://falabella-my.sharepoint.com/personal/mbsalasc_tottus_cl/Documents/Escritorio/Developer/Automatismo/Automatizaciones/Cancelar task/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{EAF8509C-23FA-4493-A943-466283222534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC01C131-2AAD-4683-9C0F-DE9E48ED5CE8}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{68C6D81B-7F2A-4A08-B0EE-34317DC6B7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF2BB624-8349-4648-B791-4184B0A76E76}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{75ACDD65-5A9D-421B-981C-237A89B9AE57}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7566D6F1-4243-4FBB-BAD3-7543DF3C6B4F}"/>
   </bookViews>
   <sheets>
-    <sheet name="report-1769714763037" sheetId="1" r:id="rId1"/>
+    <sheet name="report-1769886364812" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="26">
   <si>
     <t>FECHA_DO</t>
   </si>
@@ -52,58 +52,52 @@
     <t>P7</t>
   </si>
   <si>
-    <t>RCK29D361</t>
-  </si>
-  <si>
-    <t>RCK30D481</t>
-  </si>
-  <si>
-    <t>RCK30D501</t>
-  </si>
-  <si>
-    <t>RCK30D541</t>
-  </si>
-  <si>
-    <t>RCK30D581</t>
-  </si>
-  <si>
-    <t>RCK30D621</t>
-  </si>
-  <si>
-    <t>RCK30D681</t>
-  </si>
-  <si>
-    <t>RCK30I331</t>
-  </si>
-  <si>
-    <t>RCK30I411</t>
-  </si>
-  <si>
-    <t>RCK30I431</t>
-  </si>
-  <si>
-    <t>RCK30I451</t>
-  </si>
-  <si>
-    <t>RCK30I491</t>
-  </si>
-  <si>
-    <t>RCK20D421</t>
-  </si>
-  <si>
-    <t>RCK29D781</t>
-  </si>
-  <si>
-    <t>RCK31D061</t>
-  </si>
-  <si>
-    <t>RCK31D341</t>
-  </si>
-  <si>
-    <t>RCK20D861</t>
-  </si>
-  <si>
-    <t>RCK29I571</t>
+    <t>RCK29I051</t>
+  </si>
+  <si>
+    <t>RCK29I651</t>
+  </si>
+  <si>
+    <t>RCK29D141</t>
+  </si>
+  <si>
+    <t>RCK29D201</t>
+  </si>
+  <si>
+    <t>RCK29D221</t>
+  </si>
+  <si>
+    <t>RCK29D241</t>
+  </si>
+  <si>
+    <t>RCK29I431</t>
+  </si>
+  <si>
+    <t>RCK29I471</t>
+  </si>
+  <si>
+    <t>RCK29I511</t>
+  </si>
+  <si>
+    <t>RCK29I551</t>
+  </si>
+  <si>
+    <t>P9</t>
+  </si>
+  <si>
+    <t>38I2714</t>
+  </si>
+  <si>
+    <t>38D1612</t>
+  </si>
+  <si>
+    <t>38I3118</t>
+  </si>
+  <si>
+    <t>44D0612</t>
+  </si>
+  <si>
+    <t>38D0218</t>
   </si>
 </sst>
 </file>
@@ -964,8 +958,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E8ADE28-9A8F-4D6D-9196-1D10D388FDAA}">
-  <dimension ref="A1:G19"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6534EA5-3233-49E0-BB43-75F9CB9950C3}">
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -993,7 +987,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -1002,10 +996,10 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>19092401</v>
+        <v>19406839</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
@@ -1016,7 +1010,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -1025,10 +1019,10 @@
         <v>9</v>
       </c>
       <c r="D3">
-        <v>19092362</v>
+        <v>19406847</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
@@ -1039,7 +1033,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1048,21 +1042,21 @@
         <v>9</v>
       </c>
       <c r="D4">
-        <v>19193087</v>
+        <v>19406824</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
         <v>8</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1071,10 +1065,10 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>19092381</v>
+        <v>19406826</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
         <v>8</v>
@@ -1085,7 +1079,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1094,21 +1088,21 @@
         <v>9</v>
       </c>
       <c r="D6">
-        <v>19092404</v>
+        <v>19406837</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
         <v>8</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
@@ -1117,21 +1111,21 @@
         <v>9</v>
       </c>
       <c r="D7">
-        <v>19092352</v>
+        <v>19406816</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
@@ -1140,21 +1134,21 @@
         <v>9</v>
       </c>
       <c r="D8">
-        <v>19092353</v>
+        <v>19406843</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F8" t="s">
         <v>8</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -1163,21 +1157,21 @@
         <v>9</v>
       </c>
       <c r="D9">
-        <v>19193032</v>
+        <v>19406854</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
         <v>8</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -1186,21 +1180,21 @@
         <v>9</v>
       </c>
       <c r="D10">
-        <v>19193050</v>
+        <v>19406845</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
         <v>8</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -1209,33 +1203,33 @@
         <v>9</v>
       </c>
       <c r="D11">
-        <v>19092364</v>
+        <v>19406835</v>
       </c>
       <c r="E11" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F11" t="s">
         <v>8</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D12">
-        <v>19092365</v>
+        <v>19406901</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
         <v>8</v>
@@ -1246,19 +1240,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D13">
-        <v>19092366</v>
+        <v>19406809</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F13" t="s">
         <v>8</v>
@@ -1269,19 +1263,19 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B14" t="s">
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D14">
-        <v>19092367</v>
+        <v>19406887</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F14" t="s">
         <v>8</v>
@@ -1292,19 +1286,19 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D15">
-        <v>19060897</v>
+        <v>19406893</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F15" t="s">
         <v>8</v>
@@ -1315,94 +1309,25 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
-        <v>46045</v>
+        <v>46056</v>
       </c>
       <c r="B16" t="s">
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="D16">
-        <v>19193041</v>
+        <v>19406889</v>
       </c>
       <c r="E16" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F16" t="s">
         <v>8</v>
       </c>
       <c r="G16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="1">
-        <v>46045</v>
-      </c>
-      <c r="B17" t="s">
-        <v>7</v>
-      </c>
-      <c r="C17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17">
-        <v>19092360</v>
-      </c>
-      <c r="E17" t="s">
-        <v>19</v>
-      </c>
-      <c r="F17" t="s">
-        <v>8</v>
-      </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="1">
-        <v>46045</v>
-      </c>
-      <c r="B18" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18">
-        <v>19092361</v>
-      </c>
-      <c r="E18" t="s">
-        <v>20</v>
-      </c>
-      <c r="F18" t="s">
-        <v>8</v>
-      </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="1">
-        <v>46045</v>
-      </c>
-      <c r="B19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19">
-        <v>19179510</v>
-      </c>
-      <c r="E19" t="s">
-        <v>23</v>
-      </c>
-      <c r="F19" t="s">
-        <v>8</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove Pokeball files and update cancel task and image extraction
</commit_message>
<xml_diff>
--- a/Automatismo/Automatizaciones/Cancelar task/cancel.xlsx
+++ b/Automatismo/Automatizaciones/Cancelar task/cancel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://falabella-my.sharepoint.com/personal/mbsalasc_tottus_cl/Documents/Escritorio/Developer/Automatismo/Automatizaciones/Cancelar task/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{68C6D81B-7F2A-4A08-B0EE-34317DC6B7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF2BB624-8349-4648-B791-4184B0A76E76}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{68C6D81B-7F2A-4A08-B0EE-34317DC6B7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7636EFB0-906C-44C9-99FF-E810A829DDCB}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7566D6F1-4243-4FBB-BAD3-7543DF3C6B4F}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="26">
   <si>
     <t>FECHA_DO</t>
   </si>
@@ -52,52 +52,52 @@
     <t>P7</t>
   </si>
   <si>
-    <t>RCK29I051</t>
-  </si>
-  <si>
-    <t>RCK29I651</t>
-  </si>
-  <si>
-    <t>RCK29D141</t>
-  </si>
-  <si>
-    <t>RCK29D201</t>
-  </si>
-  <si>
-    <t>RCK29D221</t>
-  </si>
-  <si>
-    <t>RCK29D241</t>
-  </si>
-  <si>
-    <t>RCK29I431</t>
-  </si>
-  <si>
-    <t>RCK29I471</t>
-  </si>
-  <si>
-    <t>RCK29I511</t>
-  </si>
-  <si>
-    <t>RCK29I551</t>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>RCK29D601</t>
+  </si>
+  <si>
+    <t>11D0819</t>
+  </si>
+  <si>
+    <t>RCK32D201</t>
+  </si>
+  <si>
+    <t>RCK32D241</t>
+  </si>
+  <si>
+    <t>RCK32D281</t>
+  </si>
+  <si>
+    <t>RCK32D521</t>
+  </si>
+  <si>
+    <t>RCK29D641</t>
+  </si>
+  <si>
+    <t>RCK29D681</t>
+  </si>
+  <si>
+    <t>RCK29D721</t>
+  </si>
+  <si>
+    <t>RCK29D741</t>
+  </si>
+  <si>
+    <t>RCK31D221</t>
+  </si>
+  <si>
+    <t>RCK31D381</t>
+  </si>
+  <si>
+    <t>RCK31D501</t>
   </si>
   <si>
     <t>P9</t>
   </si>
   <si>
-    <t>38I2714</t>
-  </si>
-  <si>
-    <t>38D1612</t>
-  </si>
-  <si>
-    <t>38I3118</t>
-  </si>
-  <si>
-    <t>44D0612</t>
-  </si>
-  <si>
-    <t>38D0218</t>
+    <t>38D3410</t>
   </si>
 </sst>
 </file>
@@ -959,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6534EA5-3233-49E0-BB43-75F9CB9950C3}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -987,30 +987,30 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2">
-        <v>19406839</v>
+        <v>19542833</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
         <v>8</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -1019,10 +1019,10 @@
         <v>9</v>
       </c>
       <c r="D3">
-        <v>19406847</v>
+        <v>19543119</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
         <v>8</v>
@@ -1033,7 +1033,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B4" t="s">
         <v>7</v>
@@ -1042,10 +1042,10 @@
         <v>9</v>
       </c>
       <c r="D4">
-        <v>19406824</v>
+        <v>19543123</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F4" t="s">
         <v>8</v>
@@ -1056,7 +1056,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -1065,21 +1065,21 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>19406826</v>
+        <v>19543127</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s">
         <v>8</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
@@ -1088,21 +1088,21 @@
         <v>9</v>
       </c>
       <c r="D6">
-        <v>19406837</v>
+        <v>19542930</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
         <v>8</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
@@ -1111,21 +1111,21 @@
         <v>9</v>
       </c>
       <c r="D7">
-        <v>19406816</v>
+        <v>19542928</v>
       </c>
       <c r="E7" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B8" t="s">
         <v>7</v>
@@ -1134,10 +1134,10 @@
         <v>9</v>
       </c>
       <c r="D8">
-        <v>19406843</v>
+        <v>19542922</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
         <v>8</v>
@@ -1148,7 +1148,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -1157,10 +1157,10 @@
         <v>9</v>
       </c>
       <c r="D9">
-        <v>19406854</v>
+        <v>19542921</v>
       </c>
       <c r="E9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F9" t="s">
         <v>8</v>
@@ -1171,7 +1171,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B10" t="s">
         <v>7</v>
@@ -1180,21 +1180,21 @@
         <v>9</v>
       </c>
       <c r="D10">
-        <v>19406845</v>
+        <v>19543084</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F10" t="s">
         <v>8</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -1203,10 +1203,10 @@
         <v>9</v>
       </c>
       <c r="D11">
-        <v>19406835</v>
+        <v>19543052</v>
       </c>
       <c r="E11" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s">
         <v>8</v>
@@ -1217,117 +1217,94 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B12" t="s">
         <v>7</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D12">
-        <v>19406901</v>
+        <v>19543047</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F12" t="s">
         <v>8</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D13">
-        <v>19406809</v>
+        <v>19543099</v>
       </c>
       <c r="E13" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="F13" t="s">
         <v>8</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B14" t="s">
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="D14">
-        <v>19406887</v>
+        <v>19542925</v>
       </c>
       <c r="E14" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F14" t="s">
         <v>8</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
-        <v>46056</v>
+        <v>46062</v>
       </c>
       <c r="B15" t="s">
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D15">
-        <v>19406893</v>
+        <v>19543159</v>
       </c>
       <c r="E15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F15" t="s">
         <v>8</v>
       </c>
       <c r="G15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="1">
-        <v>46056</v>
-      </c>
-      <c r="B16" t="s">
-        <v>7</v>
-      </c>
-      <c r="C16" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16">
-        <v>19406889</v>
-      </c>
-      <c r="E16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16" t="s">
-        <v>8</v>
-      </c>
-      <c r="G16">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>